<commit_message>
Radar 25/09 (rotina das 08:00): GTA 6 sem online no lançamento
- Nova pauta 2026-09-25-03 com etiqueta FATO/RUMOR por slide
- Fatos: declaração da Take-Two (17/09), CEO da Twitch sobre 2027 (rumor),
  31,1 mi de views do Extended Look
- Correção: 25/09/2026 é sexta, não quinta
- Etiqueta por slide (campo tag) no render

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nvp6WtLANEYZKyqJF6nTYP
</commit_message>
<xml_diff>
--- a/registro/registro.xlsx
+++ b/registro/registro.xlsx
@@ -959,25 +959,85 @@
       <c r="T4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25-03</t>
+        </is>
+      </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Reel+Carrossel</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
-      <c r="M5" s="5" t="n"/>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
-      <c r="P5" s="5" t="n"/>
-      <c r="Q5" s="5" t="n"/>
-      <c r="R5" s="5" t="n"/>
-      <c r="S5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>GTA 6 sem online no lançamento (Take-Two) + 2027? (Twitch)</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>GTA 6 vai chegar sem modo online</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>fato forte</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>portal v2</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>radar</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>Take-Two; Bloomberg via PC Gamer</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>provisória</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Faz falta online no lançamento?</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Faz falta ter online no lançamento?</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>C4 (rótulo FATO/RUMOR)</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>rascunho</t>
+        </is>
+      </c>
       <c r="T5" s="5" t="n"/>
     </row>
     <row r="6">
@@ -18326,22 +18386,48 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25-03</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="L4" s="8">
         <f>IF(COUNT(C4:K4)=0,"",SUM(C4:K4))</f>
         <v/>
       </c>
-      <c r="M4" s="5" t="n"/>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Rotina 08:00; edição = render automático</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -24203,39 +24289,107 @@
       <c r="M9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>GTA 6 sem modo online (Take-Two 17/09) + multiplayer 2027? (Twitch)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>FATO+RUMOR</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="K10" s="9">
         <f>IF(COUNT(F10:J10)=0,"",AVERAGE(F10:J10))</f>
         <v/>
       </c>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pauta (rotina 08:00)</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25-03</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Extended Look: 31,1 mi de views na Netflix</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="K11" s="9">
         <f>IF(COUNT(F11:J11)=0,"",AVERAGE(F11:J11))</f>
         <v/>
       </c>
-      <c r="L11" s="5" t="n"/>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Dado de apoio</t>
+        </is>
+      </c>
       <c r="M11" s="5" t="n"/>
     </row>
     <row r="12">
@@ -29580,14 +29734,38 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>correção</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Radar de 25/09 marcava 'quinta-feira'; 25/09/2026 é sexta. Corrigido.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Primeira execução da rotina diária do radar (08:00 BRT).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>

</xml_diff>

<commit_message>
Radar 26/09: capa da Game Informer e álbum do GTA VI
- Pautas 2026-09-26-01 (antecipação da matéria de 29/09) e 2026-09-26-02
  (Faltam 54 dias + fato do dia: GTA VI: The Album)
- Série Faltam X dias passa a ser contagem + 1 fato novo por dia
- Fatos, estado (hipótese C8, cobertura em 29/09) e registro atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nvp6WtLANEYZKyqJF6nTYP
</commit_message>
<xml_diff>
--- a/registro/registro.xlsx
+++ b/registro/registro.xlsx
@@ -1041,47 +1041,171 @@
       <c r="T5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-01</t>
+        </is>
+      </c>
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Reel+Carrossel</t>
+        </is>
+      </c>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Game Informer: capa e 12 screenshots em 29/09</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Imagens novas do GTA 6 chegam na terça</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>antecipação</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>portal v2</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>radar</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Game Informer via Push Square</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>provisória</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>Segue pra ver tudo na terça</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>O que você mais quer ver nas imagens novas?</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>rascunho</t>
+        </is>
+      </c>
       <c r="T6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-02</t>
+        </is>
+      </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>faltam-x-dias</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Reel+Carrossel</t>
+        </is>
+      </c>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 54 dias + álbum GTA VI</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 54 dias pro GTA 6</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>número</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>portal v2</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>radar</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>Rockstar/Atlantic via Yahoo</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>provisória</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Contagem regressiva todo dia</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Que artista você queria ouvir na rádio do GTA 6?</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="S7" s="5" t="inlineStr">
+        <is>
+          <t>rascunho</t>
+        </is>
+      </c>
       <c r="T7" s="5" t="n"/>
     </row>
     <row r="8">
@@ -18430,40 +18554,92 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n"/>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-01</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="L5" s="8">
         <f>IF(COUNT(C5:K5)=0,"",SUM(C5:K5))</f>
         <v/>
       </c>
-      <c r="M5" s="5" t="n"/>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Rotina 08:00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-02</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="K6" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="L6" s="8">
         <f>IF(COUNT(C6:K6)=0,"",SUM(C6:K6))</f>
         <v/>
       </c>
-      <c r="M6" s="5" t="n"/>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Rotina 08:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -24393,57 +24569,161 @@
       <c r="M11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>GTA 6 na capa da Game Informer (12 screenshots, 29/09)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="K12" s="9">
         <f>IF(COUNT(F12:J12)=0,"",AVERAGE(F12:J12))</f>
         <v/>
       </c>
-      <c r="L12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Pauta + cobertura em 29/09</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-01</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI: The Album (34 faixas, Travis Scott, CA7RIEL)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="K13" s="9">
         <f>IF(COUNT(F13:J13)=0,"",AVERAGE(F13:J13))</f>
         <v/>
       </c>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Fato do dia na série</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26-02</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Rockstar reforça: GTA VI single player; GTA Online segue</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="K14" s="9">
         <f>IF(COUNT(F14:J14)=0,"",AVERAGE(F14:J14))</f>
         <v/>
       </c>
-      <c r="L14" s="5" t="n"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Reforça a pauta 2026-09-25-03</t>
+        </is>
+      </c>
       <c r="M14" s="5" t="n"/>
     </row>
     <row r="15">
@@ -29768,9 +30048,21 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>decisão</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Série 'Faltam X dias' passa a ser contagem + 1 fato novo por dia.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>

</xml_diff>

<commit_message>
Radar 27/09 e revisão semanal 0
- Domingo sem novidades relevantes: só a série (Faltam 53 dias + Netflix)
- Correção de exagero: 'recorde na Netflix' virou 'dominou a Netflix'
- docs/revisao-semanal/2026-09-27.md: 7 pautas, 0 posts; gargalo é ativação;
  propostas de estoque atemporal e menos volume até a estreia

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nvp6WtLANEYZKyqJF6nTYP
</commit_message>
<xml_diff>
--- a/registro/registro.xlsx
+++ b/registro/registro.xlsx
@@ -1209,25 +1209,89 @@
       <c r="T7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27-01</t>
+        </is>
+      </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>faltam-x-dias</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Reel+Carrossel</t>
+        </is>
+      </c>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 53 dias + Netflix 31,1 mi</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 53 dias pro GTA 6</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>número</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>portal v2</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>radar</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Netflix Top 10 via Variety</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>provisória</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Contagem regressiva todo dia</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Você assistiu ao Extended Look?</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="S8" s="5" t="inlineStr">
+        <is>
+          <t>rascunho</t>
+        </is>
+      </c>
       <c r="T8" s="5" t="n"/>
     </row>
     <row r="9">
@@ -18642,22 +18706,48 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27-01</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="L7" s="8">
         <f>IF(COUNT(C7:K7)=0,"",SUM(C7:K7))</f>
         <v/>
       </c>
-      <c r="M7" s="5" t="n"/>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Rotina 08:00 (domingo sem novidades)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -24727,22 +24817,58 @@
       <c r="M14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 53 dias + Extended Look 31,1 mi de views</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="K15" s="9">
         <f>IF(COUNT(F15:J15)=0,"",AVERAGE(F15:J15))</f>
         <v/>
       </c>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Série (sem novidades no dia)</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27-01</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -30065,9 +30191,21 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Revisão semanal 0: 7 pautas, 0 posts. Proposta: estoque atemporal + menos volume até a estreia.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>

</xml_diff>

<commit_message>
Radar 29/09: dia da Game Informer e Faltam 51 dias
- Registra a falha da rotina de 28/09 (não concluída) e a nova regra
- Cobertura da matéria da Game Informer fica para o radar de 30/09
- Pauta 2026-09-29-01: Faltam 51 dias + Leonida é a Flórida

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nvp6WtLANEYZKyqJF6nTYP
</commit_message>
<xml_diff>
--- a/registro/registro.xlsx
+++ b/registro/registro.xlsx
@@ -1295,25 +1295,89 @@
       <c r="T8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n"/>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29-01</t>
+        </is>
+      </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>faltam-x-dias</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Reel+Carrossel</t>
+        </is>
+      </c>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
-      <c r="S9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 51 dias + Leonida/Flórida</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 51 dias pro GTA 6</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>número</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>portal v2</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>radar</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>Rockstar; Game Informer</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>provisória</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>Contagem regressiva todo dia</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>Qual parte de Leonida você quer explorar primeiro?</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="S9" s="5" t="inlineStr">
+        <is>
+          <t>rascunho</t>
+        </is>
+      </c>
       <c r="T9" s="5" t="n"/>
     </row>
     <row r="10">
@@ -18750,22 +18814,48 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29-01</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="K8" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="L8" s="8">
         <f>IF(COUNT(C8:K8)=0,"",SUM(C8:K8))</f>
         <v/>
       </c>
-      <c r="M8" s="5" t="n"/>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Rotina 08:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -24871,40 +24961,108 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Matéria da Game Informer sai hoje (conteúdo às 11h–14h BRT)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>5</v>
+      </c>
       <c r="K16" s="9">
         <f>IF(COUNT(F16:J16)=0,"",AVERAGE(F16:J16))</f>
         <v/>
       </c>
-      <c r="L16" s="5" t="n"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Cobrir em 30/09</t>
+        </is>
+      </c>
       <c r="M16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Faltam 51 dias + Leonida = Flórida</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>GTA VI</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>FATO</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="K17" s="9">
         <f>IF(COUNT(F17:J17)=0,"",AVERAGE(F17:J17))</f>
         <v/>
       </c>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Série</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29-01</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -30208,14 +30366,38 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>correção</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Rotina de 28/09 não concluída (sem radar nem mensagem).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>decisão</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Dono recusou a checagem extra da tarde; Game Informer coberta em 30/09.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>

</xml_diff>